<commit_message>
Update corrected 2024 AQI source files
</commit_message>
<xml_diff>
--- a/aqi_target/2024/AQI_Data_City_Level_Delhi_April_2024_Hourly.xlsx
+++ b/aqi_target/2024/AQI_Data_City_Level_Delhi_April_2024_Hourly.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AQI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,122 +436,122 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>01:00:00</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>03:00</t>
+          <t>03:00:00</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>04:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>05:00</t>
+          <t>05:00:00</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>07:00:00</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>09:00:00</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>11:00:00</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>15:00:00</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>16:00:00</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:00:00</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>20:00:00</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:00:00</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:00:00</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>23:00:00</t>
         </is>
       </c>
     </row>
@@ -560,76 +560,76 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
+        <v>206</v>
+      </c>
+      <c r="C2" t="n">
+        <v>195</v>
+      </c>
+      <c r="D2" t="n">
+        <v>187</v>
+      </c>
+      <c r="E2" t="n">
+        <v>178</v>
+      </c>
+      <c r="F2" t="n">
+        <v>172</v>
+      </c>
+      <c r="G2" t="n">
+        <v>166</v>
+      </c>
+      <c r="H2" t="n">
+        <v>161</v>
+      </c>
+      <c r="I2" t="n">
+        <v>157</v>
+      </c>
+      <c r="J2" t="n">
+        <v>153</v>
+      </c>
+      <c r="K2" t="n">
         <v>148</v>
       </c>
-      <c r="C2" t="n">
-        <v>146</v>
-      </c>
-      <c r="D2" t="n">
-        <v>144</v>
-      </c>
-      <c r="E2" t="n">
-        <v>142</v>
-      </c>
-      <c r="F2" t="n">
-        <v>140</v>
-      </c>
-      <c r="G2" t="n">
-        <v>138</v>
-      </c>
-      <c r="H2" t="n">
-        <v>138</v>
-      </c>
-      <c r="I2" t="n">
-        <v>137</v>
-      </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
+        <v>143</v>
+      </c>
+      <c r="M2" t="n">
+        <v>139</v>
+      </c>
+      <c r="N2" t="n">
         <v>136</v>
       </c>
-      <c r="K2" t="n">
-        <v>136</v>
-      </c>
-      <c r="L2" t="n">
-        <v>136</v>
-      </c>
-      <c r="M2" t="n">
-        <v>140</v>
-      </c>
-      <c r="N2" t="n">
-        <v>147</v>
-      </c>
       <c r="O2" t="n">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="P2" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="Q2" t="n">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="R2" t="n">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="S2" t="n">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="T2" t="n">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="U2" t="n">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="V2" t="n">
-        <v>151</v>
+        <v>131</v>
       </c>
       <c r="W2" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="X2" t="n">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="Y2" t="n">
-        <v>156</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3">
@@ -637,74 +637,76 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>161</v>
+        <v>130</v>
       </c>
       <c r="C3" t="n">
-        <v>165</v>
+        <v>130</v>
       </c>
       <c r="D3" t="n">
-        <v>169</v>
+        <v>132</v>
       </c>
       <c r="E3" t="n">
-        <v>171</v>
+        <v>133</v>
       </c>
       <c r="F3" t="n">
-        <v>178</v>
+        <v>135</v>
       </c>
       <c r="G3" t="n">
-        <v>182</v>
+        <v>136</v>
       </c>
       <c r="H3" t="n">
-        <v>186</v>
+        <v>137</v>
       </c>
       <c r="I3" t="n">
-        <v>191</v>
+        <v>139</v>
       </c>
       <c r="J3" t="n">
-        <v>195</v>
+        <v>141</v>
       </c>
       <c r="K3" t="n">
-        <v>199</v>
+        <v>143</v>
       </c>
       <c r="L3" t="n">
-        <v>205</v>
+        <v>143</v>
       </c>
       <c r="M3" t="n">
-        <v>210</v>
+        <v>143</v>
       </c>
       <c r="N3" t="n">
-        <v>219</v>
+        <v>145</v>
       </c>
       <c r="O3" t="n">
-        <v>219</v>
+        <v>144</v>
       </c>
       <c r="P3" t="n">
-        <v>221</v>
+        <v>145</v>
       </c>
       <c r="Q3" t="n">
-        <v>216</v>
+        <v>143</v>
       </c>
       <c r="R3" t="n">
-        <v>217</v>
+        <v>144</v>
       </c>
       <c r="S3" t="n">
-        <v>212</v>
+        <v>145</v>
       </c>
       <c r="T3" t="n">
-        <v>210</v>
-      </c>
-      <c r="U3" t="inlineStr"/>
+        <v>145</v>
+      </c>
+      <c r="U3" t="n">
+        <v>145</v>
+      </c>
       <c r="V3" t="n">
-        <v>210</v>
+        <v>146</v>
       </c>
       <c r="W3" t="n">
-        <v>215</v>
+        <v>146</v>
       </c>
       <c r="X3" t="n">
-        <v>215</v>
+        <v>146</v>
       </c>
       <c r="Y3" t="n">
-        <v>220</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4">
@@ -712,74 +714,76 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>223</v>
+        <v>150</v>
       </c>
       <c r="C4" t="n">
-        <v>226</v>
+        <v>151</v>
       </c>
       <c r="D4" t="n">
-        <v>228</v>
+        <v>153</v>
       </c>
       <c r="E4" t="n">
-        <v>228</v>
+        <v>154</v>
       </c>
       <c r="F4" t="n">
-        <v>228</v>
+        <v>156</v>
       </c>
       <c r="G4" t="n">
-        <v>228</v>
+        <v>157</v>
       </c>
       <c r="H4" t="n">
-        <v>226</v>
+        <v>158</v>
       </c>
       <c r="I4" t="n">
-        <v>222</v>
+        <v>157</v>
       </c>
       <c r="J4" t="n">
-        <v>219</v>
+        <v>157</v>
       </c>
       <c r="K4" t="n">
-        <v>216</v>
+        <v>156</v>
       </c>
       <c r="L4" t="n">
-        <v>214</v>
+        <v>159</v>
       </c>
       <c r="M4" t="n">
-        <v>214</v>
+        <v>163</v>
       </c>
       <c r="N4" t="n">
-        <v>217</v>
-      </c>
-      <c r="O4" t="inlineStr"/>
+        <v>171</v>
+      </c>
+      <c r="O4" t="n">
+        <v>176</v>
+      </c>
       <c r="P4" t="n">
-        <v>224</v>
+        <v>175</v>
       </c>
       <c r="Q4" t="n">
-        <v>217</v>
+        <v>168</v>
       </c>
       <c r="R4" t="n">
-        <v>217</v>
+        <v>167</v>
       </c>
       <c r="S4" t="n">
-        <v>212</v>
+        <v>170</v>
       </c>
       <c r="T4" t="n">
-        <v>211</v>
+        <v>167</v>
       </c>
       <c r="U4" t="n">
-        <v>208</v>
+        <v>169</v>
       </c>
       <c r="V4" t="n">
-        <v>209</v>
+        <v>167</v>
       </c>
       <c r="W4" t="n">
-        <v>210</v>
+        <v>168</v>
       </c>
       <c r="X4" t="n">
-        <v>210</v>
+        <v>171</v>
       </c>
       <c r="Y4" t="n">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5">
@@ -787,74 +791,76 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>204</v>
+        <v>179</v>
       </c>
       <c r="C5" t="n">
-        <v>204</v>
+        <v>183</v>
       </c>
       <c r="D5" t="n">
-        <v>205</v>
+        <v>186</v>
       </c>
       <c r="E5" t="n">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="F5" t="n">
-        <v>208</v>
+        <v>190</v>
       </c>
       <c r="G5" t="n">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="H5" t="n">
-        <v>210</v>
+        <v>183</v>
       </c>
       <c r="I5" t="n">
-        <v>211</v>
+        <v>181</v>
       </c>
       <c r="J5" t="n">
-        <v>212</v>
+        <v>179</v>
       </c>
       <c r="K5" t="n">
-        <v>216</v>
+        <v>177</v>
       </c>
       <c r="L5" t="n">
-        <v>216</v>
+        <v>176</v>
       </c>
       <c r="M5" t="n">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="N5" t="n">
-        <v>227</v>
+        <v>177</v>
       </c>
       <c r="O5" t="n">
-        <v>225</v>
+        <v>178</v>
       </c>
       <c r="P5" t="n">
-        <v>224</v>
+        <v>178</v>
       </c>
       <c r="Q5" t="n">
-        <v>220</v>
+        <v>179</v>
       </c>
       <c r="R5" t="n">
-        <v>219</v>
+        <v>173</v>
       </c>
       <c r="S5" t="n">
-        <v>220</v>
+        <v>171</v>
       </c>
       <c r="T5" t="n">
-        <v>221</v>
+        <v>171</v>
       </c>
       <c r="U5" t="n">
-        <v>222</v>
+        <v>170</v>
       </c>
       <c r="V5" t="n">
-        <v>222</v>
+        <v>167</v>
       </c>
       <c r="W5" t="n">
-        <v>218</v>
-      </c>
-      <c r="X5" t="inlineStr"/>
+        <v>166</v>
+      </c>
+      <c r="X5" t="n">
+        <v>166</v>
+      </c>
       <c r="Y5" t="n">
-        <v>216</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6">
@@ -862,76 +868,76 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>208</v>
+        <v>166</v>
       </c>
       <c r="C6" t="n">
-        <v>201</v>
+        <v>165</v>
       </c>
       <c r="D6" t="n">
-        <v>197</v>
+        <v>163</v>
       </c>
       <c r="E6" t="n">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="F6" t="n">
-        <v>190</v>
+        <v>162</v>
       </c>
       <c r="G6" t="n">
-        <v>182</v>
+        <v>163</v>
       </c>
       <c r="H6" t="n">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="I6" t="n">
+        <v>167</v>
+      </c>
+      <c r="J6" t="n">
+        <v>169</v>
+      </c>
+      <c r="K6" t="n">
+        <v>169</v>
+      </c>
+      <c r="L6" t="n">
+        <v>168</v>
+      </c>
+      <c r="M6" t="n">
+        <v>168</v>
+      </c>
+      <c r="N6" t="n">
+        <v>168</v>
+      </c>
+      <c r="O6" t="n">
+        <v>169</v>
+      </c>
+      <c r="P6" t="n">
+        <v>172</v>
+      </c>
+      <c r="Q6" t="n">
         <v>173</v>
       </c>
-      <c r="J6" t="n">
+      <c r="R6" t="n">
         <v>174</v>
       </c>
-      <c r="K6" t="n">
-        <v>164</v>
-      </c>
-      <c r="L6" t="n">
-        <v>160</v>
-      </c>
-      <c r="M6" t="n">
-        <v>164</v>
-      </c>
-      <c r="N6" t="n">
-        <v>170</v>
-      </c>
-      <c r="O6" t="n">
-        <v>168</v>
-      </c>
-      <c r="P6" t="n">
-        <v>167</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>164</v>
-      </c>
-      <c r="R6" t="n">
-        <v>163</v>
-      </c>
       <c r="S6" t="n">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="T6" t="n">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="U6" t="n">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="V6" t="n">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="W6" t="n">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="X6" t="n">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="Y6" t="n">
-        <v>160</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7">
@@ -939,76 +945,76 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C7" t="n">
+        <v>164</v>
+      </c>
+      <c r="D7" t="n">
+        <v>163</v>
+      </c>
+      <c r="E7" t="n">
+        <v>163</v>
+      </c>
+      <c r="F7" t="n">
+        <v>164</v>
+      </c>
+      <c r="G7" t="n">
         <v>165</v>
       </c>
-      <c r="D7" t="n">
+      <c r="H7" t="n">
+        <v>165</v>
+      </c>
+      <c r="I7" t="n">
+        <v>166</v>
+      </c>
+      <c r="J7" t="n">
+        <v>166</v>
+      </c>
+      <c r="K7" t="n">
+        <v>168</v>
+      </c>
+      <c r="L7" t="n">
         <v>169</v>
       </c>
-      <c r="E7" t="n">
+      <c r="M7" t="n">
+        <v>171</v>
+      </c>
+      <c r="N7" t="n">
         <v>173</v>
       </c>
-      <c r="F7" t="n">
-        <v>177</v>
-      </c>
-      <c r="G7" t="n">
-        <v>183</v>
-      </c>
-      <c r="H7" t="n">
-        <v>189</v>
-      </c>
-      <c r="I7" t="n">
-        <v>194</v>
-      </c>
-      <c r="J7" t="n">
-        <v>198</v>
-      </c>
-      <c r="K7" t="n">
-        <v>198</v>
-      </c>
-      <c r="L7" t="n">
-        <v>198</v>
-      </c>
-      <c r="M7" t="n">
-        <v>204</v>
-      </c>
-      <c r="N7" t="n">
-        <v>216</v>
-      </c>
       <c r="O7" t="n">
-        <v>218</v>
+        <v>173</v>
       </c>
       <c r="P7" t="n">
-        <v>218</v>
+        <v>170</v>
       </c>
       <c r="Q7" t="n">
-        <v>209</v>
+        <v>169</v>
       </c>
       <c r="R7" t="n">
-        <v>209</v>
+        <v>168</v>
       </c>
       <c r="S7" t="n">
-        <v>203</v>
+        <v>169</v>
       </c>
       <c r="T7" t="n">
-        <v>201</v>
+        <v>166</v>
       </c>
       <c r="U7" t="n">
-        <v>202</v>
+        <v>167</v>
       </c>
       <c r="V7" t="n">
-        <v>202</v>
+        <v>165</v>
       </c>
       <c r="W7" t="n">
-        <v>201</v>
+        <v>163</v>
       </c>
       <c r="X7" t="n">
-        <v>201</v>
+        <v>161</v>
       </c>
       <c r="Y7" t="n">
-        <v>203</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8">
@@ -1016,76 +1022,76 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>206</v>
+        <v>159</v>
       </c>
       <c r="C8" t="n">
-        <v>206</v>
+        <v>161</v>
       </c>
       <c r="D8" t="n">
-        <v>210</v>
+        <v>161</v>
       </c>
       <c r="E8" t="n">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="F8" t="n">
-        <v>220</v>
+        <v>162</v>
       </c>
       <c r="G8" t="n">
-        <v>222</v>
+        <v>164</v>
       </c>
       <c r="H8" t="n">
-        <v>224</v>
+        <v>167</v>
       </c>
       <c r="I8" t="n">
-        <v>224</v>
+        <v>170</v>
       </c>
       <c r="J8" t="n">
-        <v>225</v>
+        <v>173</v>
       </c>
       <c r="K8" t="n">
-        <v>230</v>
+        <v>176</v>
       </c>
       <c r="L8" t="n">
-        <v>237</v>
+        <v>179</v>
       </c>
       <c r="M8" t="n">
-        <v>239</v>
+        <v>184</v>
       </c>
       <c r="N8" t="n">
-        <v>250</v>
+        <v>184</v>
       </c>
       <c r="O8" t="n">
-        <v>254</v>
+        <v>182</v>
       </c>
       <c r="P8" t="n">
-        <v>254</v>
+        <v>181</v>
       </c>
       <c r="Q8" t="n">
-        <v>260</v>
+        <v>180</v>
       </c>
       <c r="R8" t="n">
-        <v>261</v>
+        <v>179</v>
       </c>
       <c r="S8" t="n">
-        <v>264</v>
+        <v>177</v>
       </c>
       <c r="T8" t="n">
-        <v>259</v>
+        <v>174</v>
       </c>
       <c r="U8" t="n">
-        <v>259</v>
+        <v>173</v>
       </c>
       <c r="V8" t="n">
-        <v>256</v>
+        <v>173</v>
       </c>
       <c r="W8" t="n">
-        <v>254</v>
+        <v>173</v>
       </c>
       <c r="X8" t="n">
-        <v>251</v>
+        <v>174</v>
       </c>
       <c r="Y8" t="n">
-        <v>251</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9">
@@ -1093,76 +1099,76 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>250</v>
+        <v>179</v>
       </c>
       <c r="C9" t="n">
-        <v>248</v>
+        <v>181</v>
       </c>
       <c r="D9" t="n">
-        <v>246</v>
+        <v>182</v>
       </c>
       <c r="E9" t="n">
-        <v>238</v>
+        <v>183</v>
       </c>
       <c r="F9" t="n">
-        <v>236</v>
+        <v>182</v>
       </c>
       <c r="G9" t="n">
-        <v>233</v>
+        <v>182</v>
       </c>
       <c r="H9" t="n">
-        <v>228</v>
+        <v>180</v>
       </c>
       <c r="I9" t="n">
-        <v>224</v>
+        <v>179</v>
       </c>
       <c r="J9" t="n">
-        <v>221</v>
+        <v>182</v>
       </c>
       <c r="K9" t="n">
-        <v>216</v>
+        <v>182</v>
       </c>
       <c r="L9" t="n">
-        <v>214</v>
+        <v>184</v>
       </c>
       <c r="M9" t="n">
-        <v>214</v>
+        <v>188</v>
       </c>
       <c r="N9" t="n">
-        <v>222</v>
+        <v>192</v>
       </c>
       <c r="O9" t="n">
-        <v>229</v>
+        <v>192</v>
       </c>
       <c r="P9" t="n">
-        <v>234</v>
+        <v>191</v>
       </c>
       <c r="Q9" t="n">
-        <v>237</v>
+        <v>191</v>
       </c>
       <c r="R9" t="n">
-        <v>243</v>
+        <v>191</v>
       </c>
       <c r="S9" t="n">
-        <v>244</v>
+        <v>191</v>
       </c>
       <c r="T9" t="n">
-        <v>236</v>
+        <v>194</v>
       </c>
       <c r="U9" t="n">
-        <v>238</v>
+        <v>194</v>
       </c>
       <c r="V9" t="n">
-        <v>236</v>
+        <v>192</v>
       </c>
       <c r="W9" t="n">
-        <v>237</v>
+        <v>193</v>
       </c>
       <c r="X9" t="n">
-        <v>238</v>
+        <v>193</v>
       </c>
       <c r="Y9" t="n">
-        <v>237</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10">
@@ -1170,74 +1176,76 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>235</v>
+        <v>191</v>
       </c>
       <c r="C10" t="n">
-        <v>234</v>
+        <v>191</v>
       </c>
       <c r="D10" t="n">
-        <v>234</v>
+        <v>190</v>
       </c>
       <c r="E10" t="n">
-        <v>232</v>
+        <v>191</v>
       </c>
       <c r="F10" t="n">
-        <v>232</v>
+        <v>191</v>
       </c>
       <c r="G10" t="n">
-        <v>231</v>
+        <v>192</v>
       </c>
       <c r="H10" t="n">
-        <v>232</v>
+        <v>192</v>
       </c>
       <c r="I10" t="n">
-        <v>231</v>
+        <v>192</v>
       </c>
       <c r="J10" t="n">
-        <v>232</v>
+        <v>191</v>
       </c>
       <c r="K10" t="n">
-        <v>231</v>
+        <v>185</v>
       </c>
       <c r="L10" t="n">
-        <v>232</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
+        <v>184</v>
+      </c>
+      <c r="M10" t="n">
+        <v>187</v>
+      </c>
       <c r="N10" t="n">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="O10" t="n">
-        <v>236</v>
+        <v>204</v>
       </c>
       <c r="P10" t="n">
-        <v>244</v>
+        <v>206</v>
       </c>
       <c r="Q10" t="n">
-        <v>244</v>
+        <v>203</v>
       </c>
       <c r="R10" t="n">
-        <v>246</v>
+        <v>203</v>
       </c>
       <c r="S10" t="n">
-        <v>249</v>
+        <v>201</v>
       </c>
       <c r="T10" t="n">
-        <v>239</v>
+        <v>198</v>
       </c>
       <c r="U10" t="n">
-        <v>233</v>
+        <v>201</v>
       </c>
       <c r="V10" t="n">
-        <v>231</v>
+        <v>197</v>
       </c>
       <c r="W10" t="n">
-        <v>235</v>
+        <v>198</v>
       </c>
       <c r="X10" t="n">
-        <v>234</v>
+        <v>192</v>
       </c>
       <c r="Y10" t="n">
-        <v>234</v>
+        <v>191</v>
       </c>
     </row>
     <row r="11">
@@ -1245,76 +1253,76 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>234</v>
+        <v>191</v>
       </c>
       <c r="C11" t="n">
-        <v>235</v>
+        <v>193</v>
       </c>
       <c r="D11" t="n">
-        <v>235</v>
+        <v>195</v>
       </c>
       <c r="E11" t="n">
-        <v>236</v>
+        <v>199</v>
       </c>
       <c r="F11" t="n">
-        <v>238</v>
+        <v>200</v>
       </c>
       <c r="G11" t="n">
-        <v>238</v>
+        <v>200</v>
       </c>
       <c r="H11" t="n">
-        <v>238</v>
+        <v>202</v>
       </c>
       <c r="I11" t="n">
-        <v>238</v>
+        <v>202</v>
       </c>
       <c r="J11" t="n">
-        <v>240</v>
+        <v>203</v>
       </c>
       <c r="K11" t="n">
-        <v>242</v>
+        <v>204</v>
       </c>
       <c r="L11" t="n">
-        <v>244</v>
+        <v>206</v>
       </c>
       <c r="M11" t="n">
-        <v>246</v>
+        <v>209</v>
       </c>
       <c r="N11" t="n">
-        <v>251</v>
+        <v>221</v>
       </c>
       <c r="O11" t="n">
-        <v>250</v>
+        <v>223</v>
       </c>
       <c r="P11" t="n">
-        <v>257</v>
+        <v>218</v>
       </c>
       <c r="Q11" t="n">
-        <v>259</v>
+        <v>221</v>
       </c>
       <c r="R11" t="n">
-        <v>256</v>
+        <v>222</v>
       </c>
       <c r="S11" t="n">
-        <v>245</v>
+        <v>222</v>
       </c>
       <c r="T11" t="n">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="U11" t="n">
-        <v>248</v>
+        <v>223</v>
       </c>
       <c r="V11" t="n">
-        <v>249</v>
+        <v>220</v>
       </c>
       <c r="W11" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="X11" t="n">
-        <v>234</v>
+        <v>221</v>
       </c>
       <c r="Y11" t="n">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12">
@@ -1322,74 +1330,76 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C12" t="n">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="D12" t="n">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="E12" t="n">
-        <v>202</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
+        <v>221</v>
+      </c>
+      <c r="F12" t="n">
+        <v>223</v>
+      </c>
       <c r="G12" t="n">
-        <v>194</v>
+        <v>224</v>
       </c>
       <c r="H12" t="n">
-        <v>189</v>
+        <v>225</v>
       </c>
       <c r="I12" t="n">
-        <v>185</v>
+        <v>226</v>
       </c>
       <c r="J12" t="n">
-        <v>179</v>
+        <v>228</v>
       </c>
       <c r="K12" t="n">
-        <v>172</v>
+        <v>229</v>
       </c>
       <c r="L12" t="n">
-        <v>164</v>
+        <v>229</v>
       </c>
       <c r="M12" t="n">
-        <v>161</v>
+        <v>230</v>
       </c>
       <c r="N12" t="n">
-        <v>157</v>
+        <v>232</v>
       </c>
       <c r="O12" t="n">
-        <v>156</v>
+        <v>236</v>
       </c>
       <c r="P12" t="n">
-        <v>156</v>
+        <v>237</v>
       </c>
       <c r="Q12" t="n">
-        <v>154</v>
+        <v>237</v>
       </c>
       <c r="R12" t="n">
-        <v>164</v>
+        <v>240</v>
       </c>
       <c r="S12" t="n">
-        <v>162</v>
+        <v>239</v>
       </c>
       <c r="T12" t="n">
-        <v>158</v>
+        <v>233</v>
       </c>
       <c r="U12" t="n">
-        <v>150</v>
+        <v>230</v>
       </c>
       <c r="V12" t="n">
-        <v>148</v>
+        <v>228</v>
       </c>
       <c r="W12" t="n">
-        <v>150</v>
+        <v>227</v>
       </c>
       <c r="X12" t="n">
-        <v>146</v>
+        <v>227</v>
       </c>
       <c r="Y12" t="n">
-        <v>142</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13">
@@ -1397,76 +1407,76 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>137</v>
+        <v>222</v>
       </c>
       <c r="C13" t="n">
-        <v>133</v>
+        <v>220</v>
       </c>
       <c r="D13" t="n">
-        <v>129</v>
+        <v>218</v>
       </c>
       <c r="E13" t="n">
-        <v>125</v>
+        <v>215</v>
       </c>
       <c r="F13" t="n">
-        <v>123</v>
+        <v>213</v>
       </c>
       <c r="G13" t="n">
-        <v>120</v>
+        <v>213</v>
       </c>
       <c r="H13" t="n">
-        <v>119</v>
+        <v>213</v>
       </c>
       <c r="I13" t="n">
-        <v>116</v>
+        <v>213</v>
       </c>
       <c r="J13" t="n">
-        <v>119</v>
+        <v>213</v>
       </c>
       <c r="K13" t="n">
-        <v>118</v>
+        <v>213</v>
       </c>
       <c r="L13" t="n">
-        <v>117</v>
+        <v>215</v>
       </c>
       <c r="M13" t="n">
-        <v>121</v>
+        <v>225</v>
       </c>
       <c r="N13" t="n">
-        <v>127</v>
+        <v>225</v>
       </c>
       <c r="O13" t="n">
-        <v>126</v>
+        <v>226</v>
       </c>
       <c r="P13" t="n">
-        <v>157</v>
+        <v>228</v>
       </c>
       <c r="Q13" t="n">
-        <v>163</v>
+        <v>228</v>
       </c>
       <c r="R13" t="n">
-        <v>166</v>
+        <v>232</v>
       </c>
       <c r="S13" t="n">
-        <v>162</v>
+        <v>232</v>
       </c>
       <c r="T13" t="n">
-        <v>158</v>
+        <v>228</v>
       </c>
       <c r="U13" t="n">
-        <v>141</v>
+        <v>229</v>
       </c>
       <c r="V13" t="n">
-        <v>142</v>
+        <v>230</v>
       </c>
       <c r="W13" t="n">
-        <v>134</v>
+        <v>228</v>
       </c>
       <c r="X13" t="n">
-        <v>132</v>
+        <v>229</v>
       </c>
       <c r="Y13" t="n">
-        <v>125</v>
+        <v>234</v>
       </c>
     </row>
     <row r="14">
@@ -1474,76 +1484,76 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>117</v>
+        <v>238</v>
       </c>
       <c r="C14" t="n">
-        <v>109</v>
+        <v>242</v>
       </c>
       <c r="D14" t="n">
-        <v>105</v>
+        <v>244</v>
       </c>
       <c r="E14" t="n">
-        <v>105</v>
+        <v>243</v>
       </c>
       <c r="F14" t="n">
-        <v>106</v>
+        <v>245</v>
       </c>
       <c r="G14" t="n">
-        <v>106</v>
+        <v>242</v>
       </c>
       <c r="H14" t="n">
-        <v>107</v>
+        <v>238</v>
       </c>
       <c r="I14" t="n">
-        <v>108</v>
+        <v>234</v>
       </c>
       <c r="J14" t="n">
-        <v>110</v>
+        <v>229</v>
       </c>
       <c r="K14" t="n">
-        <v>113</v>
+        <v>221</v>
       </c>
       <c r="L14" t="n">
-        <v>116</v>
+        <v>214</v>
       </c>
       <c r="M14" t="n">
-        <v>137</v>
+        <v>205</v>
       </c>
       <c r="N14" t="n">
-        <v>165</v>
+        <v>202</v>
       </c>
       <c r="O14" t="n">
-        <v>176</v>
+        <v>202</v>
       </c>
       <c r="P14" t="n">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="Q14" t="n">
-        <v>169</v>
+        <v>200</v>
       </c>
       <c r="R14" t="n">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="S14" t="n">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="T14" t="n">
-        <v>166</v>
+        <v>201</v>
       </c>
       <c r="U14" t="n">
-        <v>158</v>
+        <v>200</v>
       </c>
       <c r="V14" t="n">
-        <v>158</v>
+        <v>195</v>
       </c>
       <c r="W14" t="n">
-        <v>159</v>
+        <v>190</v>
       </c>
       <c r="X14" t="n">
-        <v>144</v>
+        <v>183</v>
       </c>
       <c r="Y14" t="n">
-        <v>140</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15">
@@ -1551,76 +1561,76 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
+        <v>164</v>
+      </c>
+      <c r="C15" t="n">
+        <v>158</v>
+      </c>
+      <c r="D15" t="n">
+        <v>151</v>
+      </c>
+      <c r="E15" t="n">
+        <v>147</v>
+      </c>
+      <c r="F15" t="n">
+        <v>143</v>
+      </c>
+      <c r="G15" t="n">
         <v>141</v>
       </c>
-      <c r="C15" t="n">
-        <v>145</v>
-      </c>
-      <c r="D15" t="n">
-        <v>149</v>
-      </c>
-      <c r="E15" t="n">
-        <v>157</v>
-      </c>
-      <c r="F15" t="n">
-        <v>157</v>
-      </c>
-      <c r="G15" t="n">
-        <v>160</v>
-      </c>
       <c r="H15" t="n">
-        <v>164</v>
+        <v>140</v>
       </c>
       <c r="I15" t="n">
-        <v>168</v>
+        <v>141</v>
       </c>
       <c r="J15" t="n">
-        <v>172</v>
+        <v>134</v>
       </c>
       <c r="K15" t="n">
-        <v>174</v>
+        <v>133</v>
       </c>
       <c r="L15" t="n">
-        <v>176</v>
+        <v>134</v>
       </c>
       <c r="M15" t="n">
-        <v>179</v>
+        <v>136</v>
       </c>
       <c r="N15" t="n">
-        <v>179</v>
+        <v>138</v>
       </c>
       <c r="O15" t="n">
-        <v>196</v>
+        <v>140</v>
       </c>
       <c r="P15" t="n">
-        <v>191</v>
+        <v>142</v>
       </c>
       <c r="Q15" t="n">
-        <v>191</v>
+        <v>142</v>
       </c>
       <c r="R15" t="n">
-        <v>194</v>
+        <v>141</v>
       </c>
       <c r="S15" t="n">
-        <v>189</v>
+        <v>136</v>
       </c>
       <c r="T15" t="n">
-        <v>186</v>
+        <v>131</v>
       </c>
       <c r="U15" t="n">
-        <v>180</v>
+        <v>130</v>
       </c>
       <c r="V15" t="n">
-        <v>184</v>
+        <v>131</v>
       </c>
       <c r="W15" t="n">
-        <v>181</v>
+        <v>135</v>
       </c>
       <c r="X15" t="n">
-        <v>177</v>
+        <v>136</v>
       </c>
       <c r="Y15" t="n">
-        <v>173</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16">
@@ -1628,76 +1638,76 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="C16" t="n">
-        <v>167</v>
+        <v>147</v>
       </c>
       <c r="D16" t="n">
+        <v>152</v>
+      </c>
+      <c r="E16" t="n">
+        <v>158</v>
+      </c>
+      <c r="F16" t="n">
         <v>165</v>
       </c>
-      <c r="E16" t="n">
-        <v>164</v>
-      </c>
-      <c r="F16" t="n">
-        <v>164</v>
-      </c>
       <c r="G16" t="n">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="H16" t="n">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="I16" t="n">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="J16" t="n">
-        <v>159</v>
+        <v>192</v>
       </c>
       <c r="K16" t="n">
-        <v>159</v>
+        <v>197</v>
       </c>
       <c r="L16" t="n">
-        <v>161</v>
+        <v>200</v>
       </c>
       <c r="M16" t="n">
-        <v>162</v>
+        <v>200</v>
       </c>
       <c r="N16" t="n">
-        <v>163</v>
+        <v>203</v>
       </c>
       <c r="O16" t="n">
-        <v>165</v>
+        <v>204</v>
       </c>
       <c r="P16" t="n">
-        <v>169</v>
+        <v>200</v>
       </c>
       <c r="Q16" t="n">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="R16" t="n">
-        <v>180</v>
+        <v>205</v>
       </c>
       <c r="S16" t="n">
-        <v>176</v>
+        <v>207</v>
       </c>
       <c r="T16" t="n">
-        <v>177</v>
+        <v>206</v>
       </c>
       <c r="U16" t="n">
-        <v>170</v>
+        <v>209</v>
       </c>
       <c r="V16" t="n">
-        <v>161</v>
+        <v>209</v>
       </c>
       <c r="W16" t="n">
-        <v>161</v>
+        <v>211</v>
       </c>
       <c r="X16" t="n">
-        <v>164</v>
+        <v>214</v>
       </c>
       <c r="Y16" t="n">
-        <v>165</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17">
@@ -1705,76 +1715,76 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>165</v>
+        <v>221</v>
       </c>
       <c r="C17" t="n">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="D17" t="n">
-        <v>166</v>
+        <v>229</v>
       </c>
       <c r="E17" t="n">
-        <v>169</v>
+        <v>231</v>
       </c>
       <c r="F17" t="n">
-        <v>170</v>
+        <v>233</v>
       </c>
       <c r="G17" t="n">
-        <v>171</v>
+        <v>236</v>
       </c>
       <c r="H17" t="n">
-        <v>172</v>
+        <v>238</v>
       </c>
       <c r="I17" t="n">
-        <v>174</v>
+        <v>241</v>
       </c>
       <c r="J17" t="n">
-        <v>177</v>
+        <v>243</v>
       </c>
       <c r="K17" t="n">
-        <v>181</v>
+        <v>244</v>
       </c>
       <c r="L17" t="n">
-        <v>183</v>
+        <v>242</v>
       </c>
       <c r="M17" t="n">
-        <v>184</v>
+        <v>241</v>
       </c>
       <c r="N17" t="n">
-        <v>188</v>
+        <v>240</v>
       </c>
       <c r="O17" t="n">
-        <v>199</v>
+        <v>237</v>
       </c>
       <c r="P17" t="n">
-        <v>208</v>
+        <v>234</v>
       </c>
       <c r="Q17" t="n">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="R17" t="n">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="S17" t="n">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="T17" t="n">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="U17" t="n">
-        <v>199</v>
+        <v>225</v>
       </c>
       <c r="V17" t="n">
-        <v>203</v>
+        <v>223</v>
       </c>
       <c r="W17" t="n">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="X17" t="n">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="Y17" t="n">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="18">
@@ -1785,73 +1795,73 @@
         <v>201</v>
       </c>
       <c r="C18" t="n">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="D18" t="n">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="E18" t="n">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="F18" t="n">
-        <v>190</v>
+        <v>173</v>
       </c>
       <c r="G18" t="n">
-        <v>192</v>
+        <v>167</v>
       </c>
       <c r="H18" t="n">
-        <v>194</v>
+        <v>160</v>
       </c>
       <c r="I18" t="n">
-        <v>194</v>
+        <v>153</v>
       </c>
       <c r="J18" t="n">
-        <v>191</v>
+        <v>147</v>
       </c>
       <c r="K18" t="n">
-        <v>187</v>
+        <v>142</v>
       </c>
       <c r="L18" t="n">
-        <v>186</v>
+        <v>138</v>
       </c>
       <c r="M18" t="n">
-        <v>187</v>
+        <v>137</v>
       </c>
       <c r="N18" t="n">
-        <v>189</v>
+        <v>137</v>
       </c>
       <c r="O18" t="n">
-        <v>189</v>
+        <v>139</v>
       </c>
       <c r="P18" t="n">
-        <v>193</v>
+        <v>142</v>
       </c>
       <c r="Q18" t="n">
-        <v>200</v>
+        <v>146</v>
       </c>
       <c r="R18" t="n">
-        <v>204</v>
+        <v>147</v>
       </c>
       <c r="S18" t="n">
-        <v>206</v>
+        <v>147</v>
       </c>
       <c r="T18" t="n">
-        <v>206</v>
+        <v>146</v>
       </c>
       <c r="U18" t="n">
-        <v>195</v>
+        <v>146</v>
       </c>
       <c r="V18" t="n">
-        <v>192</v>
+        <v>146</v>
       </c>
       <c r="W18" t="n">
-        <v>193</v>
+        <v>146</v>
       </c>
       <c r="X18" t="n">
-        <v>193</v>
+        <v>144</v>
       </c>
       <c r="Y18" t="n">
-        <v>195</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19">
@@ -1859,76 +1869,76 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>199</v>
+        <v>140</v>
       </c>
       <c r="C19" t="n">
-        <v>202</v>
+        <v>140</v>
       </c>
       <c r="D19" t="n">
-        <v>205</v>
+        <v>140</v>
       </c>
       <c r="E19" t="n">
-        <v>206</v>
+        <v>142</v>
       </c>
       <c r="F19" t="n">
-        <v>207</v>
+        <v>144</v>
       </c>
       <c r="G19" t="n">
-        <v>205</v>
+        <v>146</v>
       </c>
       <c r="H19" t="n">
-        <v>200</v>
+        <v>149</v>
       </c>
       <c r="I19" t="n">
-        <v>199</v>
+        <v>152</v>
       </c>
       <c r="J19" t="n">
-        <v>200</v>
+        <v>156</v>
       </c>
       <c r="K19" t="n">
-        <v>201</v>
+        <v>157</v>
       </c>
       <c r="L19" t="n">
-        <v>202</v>
+        <v>161</v>
       </c>
       <c r="M19" t="n">
-        <v>202</v>
+        <v>167</v>
       </c>
       <c r="N19" t="n">
-        <v>207</v>
+        <v>168</v>
       </c>
       <c r="O19" t="n">
-        <v>208</v>
+        <v>169</v>
       </c>
       <c r="P19" t="n">
-        <v>215</v>
+        <v>166</v>
       </c>
       <c r="Q19" t="n">
-        <v>220</v>
+        <v>164</v>
       </c>
       <c r="R19" t="n">
-        <v>219</v>
+        <v>164</v>
       </c>
       <c r="S19" t="n">
-        <v>221</v>
+        <v>162</v>
       </c>
       <c r="T19" t="n">
-        <v>216</v>
+        <v>162</v>
       </c>
       <c r="U19" t="n">
-        <v>216</v>
+        <v>162</v>
       </c>
       <c r="V19" t="n">
-        <v>217</v>
+        <v>162</v>
       </c>
       <c r="W19" t="n">
-        <v>217</v>
+        <v>164</v>
       </c>
       <c r="X19" t="n">
-        <v>214</v>
+        <v>166</v>
       </c>
       <c r="Y19" t="n">
-        <v>212</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20">
@@ -1936,76 +1946,76 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>204</v>
+        <v>167</v>
       </c>
       <c r="C20" t="n">
-        <v>194</v>
+        <v>169</v>
       </c>
       <c r="D20" t="n">
+        <v>171</v>
+      </c>
+      <c r="E20" t="n">
+        <v>172</v>
+      </c>
+      <c r="F20" t="n">
+        <v>173</v>
+      </c>
+      <c r="G20" t="n">
+        <v>174</v>
+      </c>
+      <c r="H20" t="n">
+        <v>175</v>
+      </c>
+      <c r="I20" t="n">
+        <v>175</v>
+      </c>
+      <c r="J20" t="n">
+        <v>175</v>
+      </c>
+      <c r="K20" t="n">
+        <v>177</v>
+      </c>
+      <c r="L20" t="n">
+        <v>178</v>
+      </c>
+      <c r="M20" t="n">
+        <v>180</v>
+      </c>
+      <c r="N20" t="n">
+        <v>181</v>
+      </c>
+      <c r="O20" t="n">
+        <v>184</v>
+      </c>
+      <c r="P20" t="n">
+        <v>185</v>
+      </c>
+      <c r="Q20" t="n">
         <v>186</v>
       </c>
-      <c r="E20" t="n">
-        <v>180</v>
-      </c>
-      <c r="F20" t="n">
-        <v>175</v>
-      </c>
-      <c r="G20" t="n">
-        <v>171</v>
-      </c>
-      <c r="H20" t="n">
-        <v>168</v>
-      </c>
-      <c r="I20" t="n">
-        <v>166</v>
-      </c>
-      <c r="J20" t="n">
-        <v>164</v>
-      </c>
-      <c r="K20" t="n">
-        <v>162</v>
-      </c>
-      <c r="L20" t="n">
-        <v>161</v>
-      </c>
-      <c r="M20" t="n">
-        <v>161</v>
-      </c>
-      <c r="N20" t="n">
-        <v>161</v>
-      </c>
-      <c r="O20" t="n">
-        <v>161</v>
-      </c>
-      <c r="P20" t="n">
-        <v>162</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>163</v>
-      </c>
       <c r="R20" t="n">
-        <v>165</v>
+        <v>186</v>
       </c>
       <c r="S20" t="n">
-        <v>166</v>
+        <v>186</v>
       </c>
       <c r="T20" t="n">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="U20" t="n">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="V20" t="n">
-        <v>165</v>
+        <v>187</v>
       </c>
       <c r="W20" t="n">
-        <v>156</v>
+        <v>187</v>
       </c>
       <c r="X20" t="n">
-        <v>150</v>
+        <v>189</v>
       </c>
       <c r="Y20" t="n">
-        <v>143</v>
+        <v>193</v>
       </c>
     </row>
     <row r="21">
@@ -2013,76 +2023,76 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>143</v>
+        <v>200</v>
       </c>
       <c r="C21" t="n">
-        <v>145</v>
+        <v>210</v>
       </c>
       <c r="D21" t="n">
-        <v>146</v>
+        <v>215</v>
       </c>
       <c r="E21" t="n">
-        <v>148</v>
+        <v>222</v>
       </c>
       <c r="F21" t="n">
-        <v>149</v>
+        <v>224</v>
       </c>
       <c r="G21" t="n">
-        <v>150</v>
+        <v>223</v>
       </c>
       <c r="H21" t="n">
-        <v>151</v>
+        <v>221</v>
       </c>
       <c r="I21" t="n">
-        <v>150</v>
+        <v>220</v>
       </c>
       <c r="J21" t="n">
-        <v>149</v>
+        <v>221</v>
       </c>
       <c r="K21" t="n">
-        <v>147</v>
+        <v>220</v>
       </c>
       <c r="L21" t="n">
-        <v>146</v>
+        <v>217</v>
       </c>
       <c r="M21" t="n">
-        <v>144</v>
+        <v>215</v>
       </c>
       <c r="N21" t="n">
-        <v>143</v>
+        <v>213</v>
       </c>
       <c r="O21" t="n">
-        <v>143</v>
+        <v>214</v>
       </c>
       <c r="P21" t="n">
-        <v>144</v>
+        <v>216</v>
       </c>
       <c r="Q21" t="n">
-        <v>141</v>
+        <v>218</v>
       </c>
       <c r="R21" t="n">
-        <v>140</v>
+        <v>219</v>
       </c>
       <c r="S21" t="n">
-        <v>139</v>
+        <v>220</v>
       </c>
       <c r="T21" t="n">
-        <v>138</v>
+        <v>220</v>
       </c>
       <c r="U21" t="n">
-        <v>137</v>
+        <v>221</v>
       </c>
       <c r="V21" t="n">
-        <v>138</v>
+        <v>220</v>
       </c>
       <c r="W21" t="n">
-        <v>140</v>
+        <v>218</v>
       </c>
       <c r="X21" t="n">
-        <v>141</v>
+        <v>213</v>
       </c>
       <c r="Y21" t="n">
-        <v>144</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22">
@@ -2090,76 +2100,76 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>148</v>
+        <v>199</v>
       </c>
       <c r="C22" t="n">
+        <v>191</v>
+      </c>
+      <c r="D22" t="n">
+        <v>183</v>
+      </c>
+      <c r="E22" t="n">
+        <v>176</v>
+      </c>
+      <c r="F22" t="n">
+        <v>171</v>
+      </c>
+      <c r="G22" t="n">
+        <v>168</v>
+      </c>
+      <c r="H22" t="n">
+        <v>166</v>
+      </c>
+      <c r="I22" t="n">
+        <v>163</v>
+      </c>
+      <c r="J22" t="n">
+        <v>156</v>
+      </c>
+      <c r="K22" t="n">
+        <v>150</v>
+      </c>
+      <c r="L22" t="n">
+        <v>150</v>
+      </c>
+      <c r="M22" t="n">
         <v>151</v>
       </c>
-      <c r="D22" t="n">
-        <v>155</v>
-      </c>
-      <c r="E22" t="n">
-        <v>159</v>
-      </c>
-      <c r="F22" t="n">
-        <v>162</v>
-      </c>
-      <c r="G22" t="n">
-        <v>166</v>
-      </c>
-      <c r="H22" t="n">
-        <v>169</v>
-      </c>
-      <c r="I22" t="n">
-        <v>173</v>
-      </c>
-      <c r="J22" t="n">
-        <v>177</v>
-      </c>
-      <c r="K22" t="n">
-        <v>182</v>
-      </c>
-      <c r="L22" t="n">
-        <v>187</v>
-      </c>
-      <c r="M22" t="n">
-        <v>192</v>
-      </c>
       <c r="N22" t="n">
-        <v>197</v>
+        <v>151</v>
       </c>
       <c r="O22" t="n">
-        <v>201</v>
+        <v>147</v>
       </c>
       <c r="P22" t="n">
-        <v>204</v>
+        <v>144</v>
       </c>
       <c r="Q22" t="n">
-        <v>205</v>
+        <v>140</v>
       </c>
       <c r="R22" t="n">
-        <v>205</v>
+        <v>139</v>
       </c>
       <c r="S22" t="n">
-        <v>206</v>
+        <v>139</v>
       </c>
       <c r="T22" t="n">
-        <v>206</v>
+        <v>137</v>
       </c>
       <c r="U22" t="n">
-        <v>206</v>
+        <v>134</v>
       </c>
       <c r="V22" t="n">
-        <v>206</v>
+        <v>131</v>
       </c>
       <c r="W22" t="n">
-        <v>207</v>
+        <v>130</v>
       </c>
       <c r="X22" t="n">
-        <v>209</v>
+        <v>130</v>
       </c>
       <c r="Y22" t="n">
-        <v>211</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23">
@@ -2167,76 +2177,76 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>211</v>
+        <v>132</v>
       </c>
       <c r="C23" t="n">
-        <v>212</v>
+        <v>134</v>
       </c>
       <c r="D23" t="n">
-        <v>213</v>
+        <v>136</v>
       </c>
       <c r="E23" t="n">
-        <v>214</v>
+        <v>137</v>
       </c>
       <c r="F23" t="n">
-        <v>216</v>
+        <v>141</v>
       </c>
       <c r="G23" t="n">
-        <v>218</v>
+        <v>140</v>
       </c>
       <c r="H23" t="n">
-        <v>222</v>
+        <v>139</v>
       </c>
       <c r="I23" t="n">
-        <v>225</v>
+        <v>135</v>
       </c>
       <c r="J23" t="n">
-        <v>227</v>
+        <v>132</v>
       </c>
       <c r="K23" t="n">
-        <v>229</v>
+        <v>130</v>
       </c>
       <c r="L23" t="n">
-        <v>233</v>
+        <v>128</v>
       </c>
       <c r="M23" t="n">
-        <v>234</v>
+        <v>128</v>
       </c>
       <c r="N23" t="n">
-        <v>234</v>
+        <v>130</v>
       </c>
       <c r="O23" t="n">
-        <v>230</v>
+        <v>132</v>
       </c>
       <c r="P23" t="n">
-        <v>231</v>
+        <v>132</v>
       </c>
       <c r="Q23" t="n">
-        <v>229</v>
+        <v>129</v>
       </c>
       <c r="R23" t="n">
-        <v>227</v>
+        <v>130</v>
       </c>
       <c r="S23" t="n">
-        <v>226</v>
+        <v>130</v>
       </c>
       <c r="T23" t="n">
-        <v>225</v>
+        <v>128</v>
       </c>
       <c r="U23" t="n">
-        <v>224</v>
+        <v>130</v>
       </c>
       <c r="V23" t="n">
-        <v>222</v>
+        <v>127</v>
       </c>
       <c r="W23" t="n">
-        <v>222</v>
+        <v>123</v>
       </c>
       <c r="X23" t="n">
-        <v>222</v>
+        <v>121</v>
       </c>
       <c r="Y23" t="n">
-        <v>219</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24">
@@ -2244,72 +2254,76 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>220</v>
+        <v>119</v>
       </c>
       <c r="C24" t="n">
-        <v>221</v>
+        <v>121</v>
       </c>
       <c r="D24" t="n">
-        <v>220</v>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
+        <v>124</v>
+      </c>
+      <c r="E24" t="n">
+        <v>126</v>
+      </c>
+      <c r="F24" t="n">
+        <v>125</v>
+      </c>
       <c r="G24" t="n">
-        <v>220</v>
+        <v>129</v>
       </c>
       <c r="H24" t="n">
-        <v>217</v>
+        <v>133</v>
       </c>
       <c r="I24" t="n">
-        <v>217</v>
+        <v>139</v>
       </c>
       <c r="J24" t="n">
-        <v>219</v>
+        <v>146</v>
       </c>
       <c r="K24" t="n">
-        <v>221</v>
+        <v>152</v>
       </c>
       <c r="L24" t="n">
-        <v>220</v>
+        <v>161</v>
       </c>
       <c r="M24" t="n">
-        <v>219</v>
+        <v>170</v>
       </c>
       <c r="N24" t="n">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="O24" t="n">
-        <v>222</v>
+        <v>179</v>
       </c>
       <c r="P24" t="n">
-        <v>219</v>
+        <v>181</v>
       </c>
       <c r="Q24" t="n">
-        <v>219</v>
+        <v>192</v>
       </c>
       <c r="R24" t="n">
-        <v>224</v>
+        <v>190</v>
       </c>
       <c r="S24" t="n">
-        <v>223</v>
+        <v>196</v>
       </c>
       <c r="T24" t="n">
-        <v>220</v>
+        <v>196</v>
       </c>
       <c r="U24" t="n">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="V24" t="n">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="W24" t="n">
-        <v>217</v>
+        <v>203</v>
       </c>
       <c r="X24" t="n">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="Y24" t="n">
-        <v>217</v>
+        <v>199</v>
       </c>
     </row>
     <row r="25">
@@ -2317,74 +2331,76 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>217</v>
+        <v>196</v>
       </c>
       <c r="C25" t="n">
-        <v>219</v>
+        <v>193</v>
       </c>
       <c r="D25" t="n">
-        <v>222</v>
+        <v>191</v>
       </c>
       <c r="E25" t="n">
-        <v>227</v>
+        <v>191</v>
       </c>
       <c r="F25" t="n">
-        <v>231</v>
+        <v>191</v>
       </c>
       <c r="G25" t="n">
-        <v>236</v>
+        <v>190</v>
       </c>
       <c r="H25" t="n">
-        <v>239</v>
+        <v>192</v>
       </c>
       <c r="I25" t="n">
-        <v>240</v>
+        <v>193</v>
       </c>
       <c r="J25" t="n">
-        <v>240</v>
+        <v>193</v>
       </c>
       <c r="K25" t="n">
-        <v>237</v>
+        <v>193</v>
       </c>
       <c r="L25" t="n">
-        <v>235</v>
+        <v>192</v>
       </c>
       <c r="M25" t="n">
-        <v>234</v>
+        <v>193</v>
       </c>
       <c r="N25" t="n">
-        <v>234</v>
+        <v>194</v>
       </c>
       <c r="O25" t="n">
-        <v>243</v>
+        <v>193</v>
       </c>
       <c r="P25" t="n">
-        <v>239</v>
+        <v>191</v>
       </c>
       <c r="Q25" t="n">
-        <v>238</v>
+        <v>191</v>
       </c>
       <c r="R25" t="n">
-        <v>227</v>
+        <v>178</v>
       </c>
       <c r="S25" t="n">
-        <v>226</v>
-      </c>
-      <c r="T25" t="inlineStr"/>
+        <v>172</v>
+      </c>
+      <c r="T25" t="n">
+        <v>170</v>
+      </c>
       <c r="U25" t="n">
-        <v>232</v>
+        <v>161</v>
       </c>
       <c r="V25" t="n">
-        <v>231</v>
+        <v>157</v>
       </c>
       <c r="W25" t="n">
-        <v>232</v>
+        <v>156</v>
       </c>
       <c r="X25" t="n">
-        <v>234</v>
+        <v>156</v>
       </c>
       <c r="Y25" t="n">
-        <v>236</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26">
@@ -2392,153 +2408,151 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>239</v>
+        <v>164</v>
       </c>
       <c r="C26" t="n">
-        <v>240</v>
+        <v>167</v>
       </c>
       <c r="D26" t="n">
-        <v>238</v>
+        <v>170</v>
       </c>
       <c r="E26" t="n">
-        <v>240</v>
+        <v>172</v>
       </c>
       <c r="F26" t="n">
-        <v>241</v>
+        <v>175</v>
       </c>
       <c r="G26" t="n">
-        <v>239</v>
+        <v>176</v>
       </c>
       <c r="H26" t="n">
-        <v>237</v>
+        <v>177</v>
       </c>
       <c r="I26" t="n">
-        <v>237</v>
+        <v>178</v>
       </c>
       <c r="J26" t="n">
-        <v>236</v>
+        <v>181</v>
       </c>
       <c r="K26" t="n">
-        <v>237</v>
+        <v>187</v>
       </c>
       <c r="L26" t="n">
-        <v>241</v>
+        <v>195</v>
       </c>
       <c r="M26" t="n">
-        <v>248</v>
+        <v>205</v>
       </c>
       <c r="N26" t="n">
-        <v>262</v>
+        <v>209</v>
       </c>
       <c r="O26" t="n">
-        <v>262</v>
+        <v>206</v>
       </c>
       <c r="P26" t="n">
-        <v>263</v>
+        <v>203</v>
       </c>
       <c r="Q26" t="n">
-        <v>262</v>
+        <v>200</v>
       </c>
       <c r="R26" t="n">
-        <v>258</v>
+        <v>200</v>
       </c>
       <c r="S26" t="n">
-        <v>256</v>
+        <v>198</v>
       </c>
       <c r="T26" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="U26" t="n">
-        <v>251</v>
+        <v>200</v>
       </c>
       <c r="V26" t="n">
-        <v>252</v>
+        <v>199</v>
       </c>
       <c r="W26" t="n">
-        <v>252</v>
+        <v>201</v>
       </c>
       <c r="X26" t="n">
-        <v>253</v>
+        <v>203</v>
       </c>
       <c r="Y26" t="n">
-        <v>250</v>
+        <v>203</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="n">
-        <v>247</v>
-      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="D27" t="n">
-        <v>246</v>
+        <v>205</v>
       </c>
       <c r="E27" t="n">
-        <v>245</v>
+        <v>202</v>
       </c>
       <c r="F27" t="n">
-        <v>244</v>
+        <v>202</v>
       </c>
       <c r="G27" t="n">
-        <v>244</v>
+        <v>200</v>
       </c>
       <c r="H27" t="n">
-        <v>247</v>
+        <v>199</v>
       </c>
       <c r="I27" t="n">
-        <v>250</v>
+        <v>197</v>
       </c>
       <c r="J27" t="n">
-        <v>252</v>
+        <v>195</v>
       </c>
       <c r="K27" t="n">
-        <v>252</v>
+        <v>190</v>
       </c>
       <c r="L27" t="n">
-        <v>255</v>
+        <v>186</v>
       </c>
       <c r="M27" t="n">
-        <v>261</v>
+        <v>188</v>
       </c>
       <c r="N27" t="n">
-        <v>260</v>
+        <v>194</v>
       </c>
       <c r="O27" t="n">
-        <v>255</v>
+        <v>192</v>
       </c>
       <c r="P27" t="n">
-        <v>253</v>
+        <v>196</v>
       </c>
       <c r="Q27" t="n">
-        <v>250</v>
+        <v>197</v>
       </c>
       <c r="R27" t="n">
-        <v>247</v>
+        <v>197</v>
       </c>
       <c r="S27" t="n">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="T27" t="n">
-        <v>250</v>
+        <v>198</v>
       </c>
       <c r="U27" t="n">
-        <v>257</v>
+        <v>198</v>
       </c>
       <c r="V27" t="n">
-        <v>256</v>
+        <v>198</v>
       </c>
       <c r="W27" t="n">
-        <v>254</v>
+        <v>195</v>
       </c>
       <c r="X27" t="n">
-        <v>251</v>
+        <v>190</v>
       </c>
       <c r="Y27" t="n">
-        <v>248</v>
+        <v>184</v>
       </c>
     </row>
     <row r="28">
@@ -2546,76 +2560,76 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>245</v>
+        <v>178</v>
       </c>
       <c r="C28" t="n">
-        <v>239</v>
+        <v>173</v>
       </c>
       <c r="D28" t="n">
-        <v>230</v>
+        <v>166</v>
       </c>
       <c r="E28" t="n">
-        <v>224</v>
+        <v>162</v>
       </c>
       <c r="F28" t="n">
-        <v>220</v>
+        <v>159</v>
       </c>
       <c r="G28" t="n">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="H28" t="n">
-        <v>213</v>
+        <v>154</v>
       </c>
       <c r="I28" t="n">
-        <v>212</v>
+        <v>152</v>
       </c>
       <c r="J28" t="n">
-        <v>216</v>
+        <v>149</v>
       </c>
       <c r="K28" t="n">
-        <v>216</v>
+        <v>146</v>
       </c>
       <c r="L28" t="n">
-        <v>215</v>
+        <v>147</v>
       </c>
       <c r="M28" t="n">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="N28" t="n">
-        <v>219</v>
+        <v>155</v>
       </c>
       <c r="O28" t="n">
-        <v>228</v>
+        <v>159</v>
       </c>
       <c r="P28" t="n">
-        <v>236</v>
+        <v>161</v>
       </c>
       <c r="Q28" t="n">
-        <v>239</v>
+        <v>164</v>
       </c>
       <c r="R28" t="n">
-        <v>246</v>
+        <v>165</v>
       </c>
       <c r="S28" t="n">
-        <v>241</v>
+        <v>171</v>
       </c>
       <c r="T28" t="n">
-        <v>233</v>
+        <v>175</v>
       </c>
       <c r="U28" t="n">
-        <v>226</v>
+        <v>177</v>
       </c>
       <c r="V28" t="n">
-        <v>226</v>
+        <v>179</v>
       </c>
       <c r="W28" t="n">
-        <v>228</v>
+        <v>179</v>
       </c>
       <c r="X28" t="n">
-        <v>231</v>
+        <v>182</v>
       </c>
       <c r="Y28" t="n">
-        <v>233</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29">
@@ -2623,76 +2637,76 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>236</v>
+        <v>190</v>
       </c>
       <c r="C29" t="n">
-        <v>240</v>
+        <v>192</v>
       </c>
       <c r="D29" t="n">
-        <v>243</v>
+        <v>195</v>
       </c>
       <c r="E29" t="n">
-        <v>248</v>
+        <v>196</v>
       </c>
       <c r="F29" t="n">
-        <v>252</v>
+        <v>196</v>
       </c>
       <c r="G29" t="n">
-        <v>254</v>
+        <v>195</v>
       </c>
       <c r="H29" t="n">
-        <v>252</v>
+        <v>195</v>
       </c>
       <c r="I29" t="n">
-        <v>249</v>
+        <v>195</v>
       </c>
       <c r="J29" t="n">
-        <v>247</v>
+        <v>195</v>
       </c>
       <c r="K29" t="n">
-        <v>248</v>
+        <v>195</v>
       </c>
       <c r="L29" t="n">
-        <v>248</v>
+        <v>192</v>
       </c>
       <c r="M29" t="n">
-        <v>251</v>
+        <v>186</v>
       </c>
       <c r="N29" t="n">
-        <v>252</v>
+        <v>184</v>
       </c>
       <c r="O29" t="n">
-        <v>256</v>
+        <v>185</v>
       </c>
       <c r="P29" t="n">
-        <v>255</v>
+        <v>177</v>
       </c>
       <c r="Q29" t="n">
-        <v>260</v>
+        <v>175</v>
       </c>
       <c r="R29" t="n">
-        <v>266</v>
+        <v>176</v>
       </c>
       <c r="S29" t="n">
-        <v>267</v>
+        <v>173</v>
       </c>
       <c r="T29" t="n">
-        <v>268</v>
+        <v>166</v>
       </c>
       <c r="U29" t="n">
-        <v>272</v>
+        <v>164</v>
       </c>
       <c r="V29" t="n">
-        <v>272</v>
+        <v>162</v>
       </c>
       <c r="W29" t="n">
-        <v>273</v>
+        <v>161</v>
       </c>
       <c r="X29" t="n">
-        <v>268</v>
+        <v>161</v>
       </c>
       <c r="Y29" t="n">
-        <v>267</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30">
@@ -2700,76 +2714,76 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>263</v>
+        <v>164</v>
       </c>
       <c r="C30" t="n">
-        <v>261</v>
+        <v>170</v>
       </c>
       <c r="D30" t="n">
-        <v>258</v>
+        <v>177</v>
       </c>
       <c r="E30" t="n">
-        <v>257</v>
+        <v>181</v>
       </c>
       <c r="F30" t="n">
-        <v>255</v>
+        <v>184</v>
       </c>
       <c r="G30" t="n">
-        <v>247</v>
+        <v>187</v>
       </c>
       <c r="H30" t="n">
-        <v>246</v>
+        <v>190</v>
       </c>
       <c r="I30" t="n">
-        <v>243</v>
+        <v>195</v>
       </c>
       <c r="J30" t="n">
-        <v>237</v>
+        <v>200</v>
       </c>
       <c r="K30" t="n">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="L30" t="n">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="M30" t="n">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="N30" t="n">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="O30" t="n">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="P30" t="n">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="Q30" t="n">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="R30" t="n">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="S30" t="n">
-        <v>205</v>
+        <v>231</v>
       </c>
       <c r="T30" t="n">
-        <v>202</v>
+        <v>238</v>
       </c>
       <c r="U30" t="n">
-        <v>198</v>
+        <v>240</v>
       </c>
       <c r="V30" t="n">
-        <v>194</v>
+        <v>240</v>
       </c>
       <c r="W30" t="n">
-        <v>191</v>
+        <v>238</v>
       </c>
       <c r="X30" t="n">
-        <v>188</v>
+        <v>235</v>
       </c>
       <c r="Y30" t="n">
-        <v>187</v>
+        <v>231</v>
       </c>
     </row>
     <row r="31">
@@ -2777,76 +2791,76 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>186</v>
+        <v>226</v>
       </c>
       <c r="C31" t="n">
-        <v>185</v>
+        <v>221</v>
       </c>
       <c r="D31" t="n">
-        <v>184</v>
+        <v>217</v>
       </c>
       <c r="E31" t="n">
+        <v>213</v>
+      </c>
+      <c r="F31" t="n">
+        <v>209</v>
+      </c>
+      <c r="G31" t="n">
+        <v>207</v>
+      </c>
+      <c r="H31" t="n">
+        <v>204</v>
+      </c>
+      <c r="I31" t="n">
+        <v>201</v>
+      </c>
+      <c r="J31" t="n">
+        <v>198</v>
+      </c>
+      <c r="K31" t="n">
+        <v>194</v>
+      </c>
+      <c r="L31" t="n">
+        <v>189</v>
+      </c>
+      <c r="M31" t="n">
         <v>188</v>
       </c>
-      <c r="F31" t="n">
+      <c r="N31" t="n">
+        <v>188</v>
+      </c>
+      <c r="O31" t="n">
+        <v>189</v>
+      </c>
+      <c r="P31" t="n">
+        <v>189</v>
+      </c>
+      <c r="Q31" t="n">
         <v>190</v>
       </c>
-      <c r="G31" t="n">
-        <v>190</v>
-      </c>
-      <c r="H31" t="n">
-        <v>191</v>
-      </c>
-      <c r="I31" t="n">
-        <v>192</v>
-      </c>
-      <c r="J31" t="n">
-        <v>191</v>
-      </c>
-      <c r="K31" t="n">
-        <v>190</v>
-      </c>
-      <c r="L31" t="n">
-        <v>190</v>
-      </c>
-      <c r="M31" t="n">
-        <v>190</v>
-      </c>
-      <c r="N31" t="n">
-        <v>193</v>
-      </c>
-      <c r="O31" t="n">
-        <v>197</v>
-      </c>
-      <c r="P31" t="n">
-        <v>199</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>196</v>
-      </c>
       <c r="R31" t="n">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="S31" t="n">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="T31" t="n">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="U31" t="n">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="V31" t="n">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="W31" t="n">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="X31" t="n">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="Y31" t="n">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>